<commit_message>
Testes finalizados com state, icon e notification
</commit_message>
<xml_diff>
--- a/Controle_Ouvidoria.xlsx
+++ b/Controle_Ouvidoria.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,239 +441,56 @@
           <t>Prazo SLA</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ID Mensagem</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>É AMANHÃ! 🎉 +R$ 1 Milhão em cupons pra você!</t>
+          <t>‎João‎ está no aguardo. Proteja a sua ofensiva dos amigos!</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Magalu</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-04-10 17:42:13</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>Duolingo</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>46130.79224537037</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>46134.625</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>000000003CD2132DFF62AC4FB33AA897F8F238EC07005E4B862F80A6B340B32A1EFF71B7518A000841023BCC00005E4B862F80A6B340B32A1EFF71B7518A0008462657BF0000</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>É AMANHÃ! 🎉 +R$ 1 Milhão em cupons pra você!</t>
+          <t>TESTE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Magalu</t>
+          <t>Robert Landim</t>
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>46122.73765046296</v>
+        <v>46130.89329861111</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>46127.61265046296</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Teste</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Robert Landim</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="n">
-        <v>46122.89899305555</v>
-      </c>
-      <c r="D4" s="1" t="n">
-        <v>46127.625</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>É AMANHÃ! 🎉 +R$ 1 Milhão em cupons pra você!</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Magalu</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>46122.73765046296</v>
-      </c>
-      <c r="D5" s="1" t="n">
-        <v>46127.61265046296</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Teste</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Robert Landim</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>46122.89899305555</v>
-      </c>
-      <c r="D6" s="1" t="n">
-        <v>46127.625</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>É AMANHÃ! 🎉 +R$ 1 Milhão em cupons pra você!</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Magalu</t>
-        </is>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>46122.73765046296</v>
-      </c>
-      <c r="D7" s="1" t="n">
-        <v>46127.61265046296</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Teste</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Robert Landim</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="n">
-        <v>46122.89899305555</v>
-      </c>
-      <c r="D8" s="1" t="n">
-        <v>46127.625</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>É AMANHÃ! 🎉 +R$ 1 Milhão em cupons pra você!</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Magalu</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="n">
-        <v>46122.73765046296</v>
-      </c>
-      <c r="D9" s="1" t="n">
-        <v>46127.61265046296</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Teste</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Robert Landim</t>
-        </is>
-      </c>
-      <c r="C10" s="1" t="n">
-        <v>46122.89899305555</v>
-      </c>
-      <c r="D10" s="1" t="n">
-        <v>46127.625</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>É AMANHÃ! 🎉 +R$ 1 Milhão em cupons pra você!</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Magalu</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="n">
-        <v>46122.73765046296</v>
-      </c>
-      <c r="D11" s="1" t="n">
-        <v>46127.61265046296</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Teste</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Robert Landim</t>
-        </is>
-      </c>
-      <c r="C12" s="1" t="n">
-        <v>46122.89899305555</v>
-      </c>
-      <c r="D12" s="1" t="n">
-        <v>46127.625</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>É AMANHÃ! 🎉 +R$ 1 Milhão em cupons pra você!</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Magalu</t>
-        </is>
-      </c>
-      <c r="C13" s="1" t="n">
-        <v>46122.73765046296</v>
-      </c>
-      <c r="D13" s="1" t="n">
-        <v>46127.61265046296</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Teste</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Robert Landim</t>
-        </is>
-      </c>
-      <c r="C14" s="1" t="n">
-        <v>46122.89899305555</v>
-      </c>
-      <c r="D14" s="1" t="n">
-        <v>46127.625</v>
+        <v>46134.625</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>000000003CD2132DFF62AC4FB33AA897F8F238EC07005E4B862F80A6B340B32A1EFF71B7518A000841023BCC00005E4B862F80A6B340B32A1EFF71B7518A0008462657C10000</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>